<commit_message>
:test_tube: Add coverage for PDF chunking with shifted merges
</commit_message>
<xml_diff>
--- a/examples/dataframe_shift/output.xlsx
+++ b/examples/dataframe_shift/output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shift Demo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Shift Demo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +31,9 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -84,7 +86,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -491,10 +493,11 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C1:D1"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A3:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:bug: Fix repeat dataframe shifting
</commit_message>
<xml_diff>
--- a/examples/dataframe_shift/output.xlsx
+++ b/examples/dataframe_shift/output.xlsx
@@ -17,13 +17,20 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -33,10 +40,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,17 +56,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE699"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFD9EAF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2F0D9"/>
+        <fgColor rgb="FFFDE9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,16 +83,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,49 +473,188 @@
   </sheetPr>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>dataframe_shift with repeat blocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Customer: Alpha Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Shift right of dataframe</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n">
+      <c r="B5" s="6" t="n">
         <v>1200</v>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Right-side merged note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Ben</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B6" s="6" t="n">
         <v>950</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Footer merged below dataframe rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+    <row r="7" ht="18" customHeight="1">
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Shift below dataframe</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Customer: Beta Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Repeat block stays aligned</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Footer follows dataframe rows</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Static footer after repeats</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="A3:C4"/>
+  <mergeCells count="5">
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>